<commit_message>
Update members.js with new member details and remove outdated entries
</commit_message>
<xml_diff>
--- a/data/members.xlsx
+++ b/data/members.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Інструкція" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Учасники'!$A$1:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Учасники'!$A$1:$G$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -539,12 +539,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Олена Коваль</t>
+          <t>Valeriia Makarenko</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Потік 2024</t>
+          <t>YouLEAD 2025</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -557,11 +557,7 @@
           <t>Україна</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>example_olena</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="3" t="n">
         <v>50.4501</v>
       </c>
@@ -572,17 +568,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Андрій Мельник</t>
+          <t>Daria Levadna</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Потік 2025</t>
+          <t>YouLEAD 2025</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Київ</t>
+          <t>Дніпро</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -590,32 +586,28 @@
           <t>Україна</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>example_andrii</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="3" t="n">
-        <v>50.4501</v>
+        <v>48.4647</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>30.5234</v>
+        <v>35.0462</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Марія Шевчук</t>
+          <t>Alisa Shcherbak</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Потік 2024</t>
+          <t>YouLEAD 2025</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Львів</t>
+          <t>Київ</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -623,251 +615,45 @@
           <t>Україна</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>example_maria</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="n"/>
       <c r="F4" s="3" t="n">
-        <v>49.8397</v>
+        <v>50.4501</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>24.0297</v>
+        <v>30.5234</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Тарас Бондар</t>
+          <t>Anastasiia Batechko</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Потік 2023</t>
+          <t>YouLEAD 2025</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Варшава</t>
+          <t>Буча</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Польща</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>example_taras</t>
-        </is>
-      </c>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
       <c r="F5" s="3" t="n">
-        <v>52.2297</v>
+        <v>50.5436</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>21.0122</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Ірина Кравчук</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Потік 2025</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Берлін</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Німеччина</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>example_iryna</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>52.52</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>13.405</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Максим Ткачук</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Потік 2023</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Лондон</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Велика Британія</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>example_maks</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>51.5072</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>-0.1276</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Софія Гриценко</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Потік 2024</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Нью-Йорк</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>США</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>example_sofia</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>40.7128</v>
-      </c>
-      <c r="G8" s="3" t="n">
-        <v>-74.006</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Данило Лисенко</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Потік 2025</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Торонто</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Канада</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>example_danylo</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>43.6532</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>-79.3832</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Катерина Павленко</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Потік 2022</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Дубай</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>ОАЕ</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>example_kate</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>25.2048</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>55.2708</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Олег Романюк</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Потік 2023</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Сінгапур</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Сінгапур</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>example_oleg</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>1.3521</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>103.8198</v>
+        <v>30.2139</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G11"/>
+  <autoFilter ref="A1:G5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -977,7 +763,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>УВАГА: дані в рядках-прикладах вигадані. Замінити їх на справжніх учасників перед публікацією.</t>
+          <t>Telegram: у колонці E впиши нік людини (без @). Поки колонка порожня, кнопка «Написати в Telegram» на картці не показується.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update members.js with new member entries and Telegram handles
</commit_message>
<xml_diff>
--- a/data/members.xlsx
+++ b/data/members.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Інструкція" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Учасники'!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Учасники'!$A$1:$G$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -557,7 +557,11 @@
           <t>Україна</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>nn1me</t>
+        </is>
+      </c>
       <c r="F2" s="3" t="n">
         <v>50.4501</v>
       </c>
@@ -586,7 +590,11 @@
           <t>Україна</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>dar_levadna</t>
+        </is>
+      </c>
       <c r="F3" s="3" t="n">
         <v>48.4647</v>
       </c>
@@ -615,7 +623,11 @@
           <t>Україна</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>ailiisaa</t>
+        </is>
+      </c>
       <c r="F4" s="3" t="n">
         <v>50.4501</v>
       </c>
@@ -644,7 +656,11 @@
           <t>Україна</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Naseqw</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="n">
         <v>50.5436</v>
       </c>
@@ -652,8 +668,998 @@
         <v>30.2139</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Pavlo Aizenberh</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2025</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Львів</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>eiissenberg</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>49.8397</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>24.0297</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Anna Bielik</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>annxq</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Kirill Horkov</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>kirillhorkov</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Stefaniia Durytska</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2025</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>streemodie</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Anya Mishchuk</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>anyamishaa</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Yeva Mohylevska</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Хмельницький</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>qrevww</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>49.423</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>26.9871</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Veronika Bondarenko</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Аліканте</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Іспанія</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>lll1va</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>38.3452</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>-0.481</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Maksym Fedorovskyi</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Maksymshark</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Oleksandr Serko</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Ковель</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>santyorik</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>51.2167</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>24.7167</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Khrystyna Shpyrka</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2025</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Відень</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Австрія</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>shpyrkaa</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>48.2082</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>16.3738</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Liza Zolotarova</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2025</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Золотурн</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Швейцарія</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>rkrx_li</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>47.2088</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>7.5372</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Mariia Bilytska</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2025</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Вінниця</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>yesimmeri</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>49.2331</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>28.4682</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Sofiko Ponomarova</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Харків</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>sowwks</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>49.9935</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>36.2304</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Maria Fedorchuk</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2025</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Хмельницький</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>maskamariyka</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>49.423</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>26.9871</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Anna Vasylieva</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2024</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Ірпінь</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>srgvnna</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>50.5218</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>30.2506</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Dmytro Baran</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2024</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Варшава</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Польща</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>dim4art</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>52.2297</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>21.0122</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Anastasiia Lavrenchuk</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2024</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>sargeryy</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Arina Bielik</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2024</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>arinabielik</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Mykhailo Dyshkant</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2024</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Братислава</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Словаччина</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>pandonn1o</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>48.1486</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>17.1077</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Yuliia Tertyshnyk</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>julkiiinss</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Artem Serebriakov</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2024</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Гельсінкі</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Фінляндія</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>artemimus</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>60.1699</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>24.9384</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Arzy Adzhibekirova</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2024</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>ArzyAdzhi</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Diana Bulai</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2025</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Світловодськ</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>dianabulai</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>49.0483</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>33.2433</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Kateryna Mysko</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Київ</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>katrinneesss</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>50.4501</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>30.5234</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Oleksandr Kachkan</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2025</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Львів</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>San3X_x</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>49.8397</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>24.0297</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Maksym Zahorodnii</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2025</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Бориспіль</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>MaximZagorodnii</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>50.3528</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>30.9553</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Mariia Hryhurko</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2024</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Одеса</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>marifxn</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>46.4825</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>30.7233</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Anastasiia Dabizha</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2024</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Одеса</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>nstsaa_a</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>46.4825</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>30.7233</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Mykola Vaskiv</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2026</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Львів</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>mykola_waskiw</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>49.8397</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>24.0297</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Anton Mazharystyi</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>YouLEAD 2022</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Братислава</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Словаччина</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>yntytyn</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>48.1486</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>17.1077</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G5"/>
+  <autoFilter ref="A1:G35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -763,7 +1769,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Telegram: у колонці E впиши нік людини (без @). Поки колонка порожня, кнопка «Написати в Telegram» на картці не показується.</t>
+          <t>Telegram: у колонці E впиши нік людини (без @). Порожня колонка — кнопка «Написати в Telegram» на картці не показується.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update members.xlsx with new member data
</commit_message>
<xml_diff>
--- a/data/members.xlsx
+++ b/data/members.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Інструкція" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Учасники'!$A$1:$G$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Учасники'!$A$1:$G$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1658,8 +1658,246 @@
         <v>17.1077</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Анастасія К</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>ankovval</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="n"/>
+      <c r="G36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Sofiia Roommate USA</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>sofkol26</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Yulian Lazutin</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Yulian_lazutin</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="n"/>
+      <c r="G38" s="3" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Hrytsenko Sofiia</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>sonfqd</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="n"/>
+      <c r="G39" s="3" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Nikolya</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Nik01ya</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="n"/>
+      <c r="G40" s="3" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>дарсі</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>reyeagama</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="n"/>
+      <c r="G41" s="3" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Anna Gorb</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>anivnaaa</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="3" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Ксюша</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>necstique</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>dashulheen</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Sofiia Novychenko</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>veinnyl</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="n"/>
+      <c r="G45" s="3" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Ivan Shuliak</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>exdreamy7</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Volodymyr Potapov</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Mo1seys</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="n"/>
+      <c r="G47" s="3" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Anastasiia Samoilovych</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Samoilovych</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="n"/>
+      <c r="G48" s="3" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>dariia</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>poriadaa</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="n"/>
+      <c r="G49" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G35"/>
+  <autoFilter ref="A1:G49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -1671,7 +1909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1725,49 +1963,56 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Рядки без міста (потік і місто ще не відомі) зберігаються тут, але на глобусі не показуються — допиши місто, і вони з'являться.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
           <t>5. Збережи файл, залишивши його в папці data/ під назвою members.xlsx.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Як дані потрапляють на сайт</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>• Щодня о 00:00 (за варшавським часом) GitHub автоматично читає цей файл і оновлює сайт.</t>
-        </is>
-      </c>
+      <c r="A12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>• Також сайт оновлюється одразу після того, як ти завантажиш нову версію файлу в репозиторій.</t>
+          <t>• Щодня о 00:00 (за варшавським часом) GitHub автоматично читає цей файл і оновлює сайт.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>• Також сайт оновлюється одразу після того, як ти завантажиш нову версію файлу в репозиторій.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t>• Рядки без імені пропускаються. Місто, яке не вдалося знайти, пропускається — воно з'явиться в журналі оновлення.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Telegram: у колонці E впиши нік людини (без @). Порожня колонка — кнопка «Написати в Telegram» на картці не показується.</t>
         </is>

</xml_diff>

<commit_message>
Implement city search functionality and update member locations in the app
</commit_message>
<xml_diff>
--- a/data/members.xlsx
+++ b/data/members.xlsx
@@ -1539,12 +1539,12 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Одеса</t>
+          <t>Філадельфія</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Україна</t>
+          <t>США</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1553,10 +1553,10 @@
         </is>
       </c>
       <c r="F32" s="3" t="n">
-        <v>46.4825</v>
+        <v>39.9526</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>30.7233</v>
+        <v>-75.1652</v>
       </c>
     </row>
     <row r="33">
@@ -1572,12 +1572,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Одеса</t>
+          <t>Нешвілл</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Україна</t>
+          <t>США</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1586,10 +1586,10 @@
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>46.4825</v>
+        <v>36.1627</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>30.7233</v>
+        <v>-86.7816</v>
       </c>
     </row>
     <row r="34">

</xml_diff>